<commit_message>
Fix sequential challenge progression in generation script
- Modified `generate_galar_paths.py` so that Sheet 2 features a strict 1-to-1 sequential unlocking process.
- Clearing Path N unlocks Path N+1.
- Fully regenerated `Galar_Paths.xlsx`.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Galar_Paths.xlsx
+++ b/Galar_Paths.xlsx
@@ -11511,7 +11511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11539,12 +11539,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Clear Route 4</t>
+          <t>Clear Route 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Unlocks Route 5</t>
+          <t>Unlocks Route 2</t>
         </is>
       </c>
     </row>
@@ -11556,12 +11556,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Clear Route 5</t>
+          <t>Clear Route 2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Unlocks Galar Mine No. 2</t>
+          <t>Unlocks Rolling Fields</t>
         </is>
       </c>
     </row>
@@ -11573,12 +11573,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Clear Galar Mine No. 2</t>
+          <t>Clear Rolling Fields</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Unlocks Motostoke Outskirts</t>
+          <t>Unlocks Dappled Grove</t>
         </is>
       </c>
     </row>
@@ -11590,12 +11590,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Clear Motostoke Outskirts</t>
+          <t>Clear Dappled Grove</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Unlocks Watchtower Ruins</t>
+          <t>Unlocks West Lake Axewell</t>
         </is>
       </c>
     </row>
@@ -11607,12 +11607,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Clear Route 6</t>
+          <t>Clear West Lake Axewell</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Unlocks Bridge Field</t>
+          <t>Unlocks East Lake Axewell</t>
         </is>
       </c>
     </row>
@@ -11624,12 +11624,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Clear Bridge Field</t>
+          <t>Clear East Lake Axewell</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Unlocks Stony Wilderness</t>
+          <t>Unlocks South Lake Miloch</t>
         </is>
       </c>
     </row>
@@ -11641,12 +11641,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Clear Glimwood Tangle</t>
+          <t>Clear South Lake Miloch</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Unlocks Route 9</t>
+          <t>Unlocks North Lake Miloch</t>
         </is>
       </c>
     </row>
@@ -11658,12 +11658,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Clear Route 9</t>
+          <t>Clear North Lake Miloch</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Unlocks Lake of Outrage</t>
+          <t>Unlocks Route 3</t>
         </is>
       </c>
     </row>
@@ -11675,12 +11675,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Clear Lake of Outrage</t>
+          <t>Clear Route 3</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Unlocks Route 10</t>
+          <t>Unlocks Galar Mine</t>
         </is>
       </c>
     </row>
@@ -11692,12 +11692,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Clear Route 10</t>
+          <t>Clear Galar Mine</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Unlocks Slumbering Weald 2</t>
+          <t>Unlocks Route 4</t>
         </is>
       </c>
     </row>
@@ -11709,333 +11709,877 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Clear Slumbering Weald 2</t>
+          <t>Clear Route 4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Unlocks Isle of Armor &amp; Crown Tundra</t>
+          <t>Unlocks Turffield Gym</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-1</t>
+          <t>Challenge 12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Clear Fields of Honor</t>
+          <t>Clear Turffield Gym</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Unlocks Soothing Wetlands</t>
+          <t>Unlocks Route 5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-2</t>
+          <t>Challenge 13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Clear Soothing Wetlands</t>
+          <t>Clear Route 5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Unlocks Forest of Focus</t>
+          <t>Unlocks Route 5 Daycare</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-3</t>
+          <t>Challenge 14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Clear Forest of Focus</t>
+          <t>Clear Route 5 Daycare</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Unlocks Challenge Beach</t>
+          <t>Unlocks Galar Mine No. 2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-4</t>
+          <t>Challenge 15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Clear Challenge Beach</t>
+          <t>Clear Galar Mine No. 2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Unlocks Brawlers' Cave</t>
+          <t>Unlocks Hulbury</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-5</t>
+          <t>Challenge 16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Clear Brawlers' Cave</t>
+          <t>Clear Hulbury</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Unlocks Challenge Road</t>
+          <t>Unlocks Hulbury Gym</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-6</t>
+          <t>Challenge 17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Clear Challenge Road</t>
+          <t>Clear Hulbury Gym</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Unlocks Training Lowlands</t>
+          <t>Unlocks Motostoke Outskirts</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-7</t>
+          <t>Challenge 18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Clear Training Lowlands</t>
+          <t>Clear Motostoke Outskirts</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Unlocks Warm-Up Tunnel</t>
+          <t>Unlocks Motostoke Gym</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-8</t>
+          <t>Challenge 19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Clear Warm-Up Tunnel</t>
+          <t>Clear Motostoke Gym</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Unlocks Workout Sea</t>
+          <t>Unlocks Watchtower Ruins</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-9</t>
+          <t>Challenge 20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Clear Workout Sea</t>
+          <t>Clear Watchtower Ruins</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Unlocks Stepping-Stone Sea</t>
+          <t>Unlocks Axew's Eye</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-10</t>
+          <t>Challenge 21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Clear Stepping-Stone Sea</t>
+          <t>Clear Axew's Eye</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Unlocks Honeycalm Island</t>
+          <t>Unlocks Slumbering Weald</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-11</t>
+          <t>Challenge 22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Clear Honeycalm Island</t>
+          <t>Clear Slumbering Weald</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Isle of Armor Completed</t>
+          <t>Unlocks Route 6</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-1</t>
+          <t>Challenge 23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Clear Slippery Slope</t>
+          <t>Clear Route 6</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Unlocks Frigid Sea</t>
+          <t>Unlocks Bridge Field Daycare</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-2</t>
+          <t>Challenge 24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Clear Frigid Sea</t>
+          <t>Clear Bridge Field Daycare</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Unlocks Roaring-Sea Caves</t>
+          <t>Unlocks Bridge Field</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-3</t>
+          <t>Challenge 25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Clear Roaring-Sea Caves</t>
+          <t>Clear Bridge Field</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Unlocks Lakeside Cave</t>
+          <t>Unlocks Stow-on-Side Gym</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-4</t>
+          <t>Challenge 26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Clear Lakeside Cave</t>
+          <t>Clear Stow-on-Side Gym</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Unlocks Old Cemetery</t>
+          <t>Unlocks Stony Wilderness</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-5</t>
+          <t>Challenge 27</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Clear Old Cemetery</t>
+          <t>Clear Stony Wilderness</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Unlocks Giant's Foot</t>
+          <t>Unlocks Dusty Bowl</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-6</t>
+          <t>Challenge 28</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Clear Giant's Foot</t>
+          <t>Clear Dusty Bowl</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Unlocks Path to the Peak</t>
+          <t>Unlocks Giant's Cap</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-7</t>
+          <t>Challenge 29</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Clear Path to the Peak</t>
+          <t>Clear Giant's Cap</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Unlocks Tunnel to the Top</t>
+          <t>Unlocks Hammerlocke Hills</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Challenge 30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Clear Hammerlocke Hills</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Unlocks Motostoke Riverbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Challenge 31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Clear Motostoke Riverbank</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Unlocks Route 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Challenge 32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Clear Route 7</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Unlocks Route 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Challenge 33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Clear Route 8</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Unlocks Glimwood Tangle</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Challenge 34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Clear Glimwood Tangle</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Unlocks Ballonlea Gym</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Challenge 35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Clear Ballonlea Gym</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Unlocks Route 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Challenge 36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Clear Route 9</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Unlocks Circhester Gym</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Challenge 37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Clear Circhester Gym</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Unlocks Lake of Outrage</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Challenge 38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Clear Lake of Outrage</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Unlocks Spikemuth Gym</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Challenge 39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Clear Spikemuth Gym</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Unlocks Route 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Challenge 40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Clear Route 10</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Unlocks Hammerlocke Gym</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Challenge 41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Clear Hammerlocke Gym</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Unlocks Slumbering Weald 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Challenge 42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Clear Slumbering Weald 2</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Unlocks Pokemon League</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Challenge 43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Clear Pokemon League</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Unlocks Isle of Armor &amp; Crown Tundra</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Clear Fields of Honor</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Unlocks Soothing Wetlands</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Clear Soothing Wetlands</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Unlocks Forest of Focus</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-3</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Clear Forest of Focus</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Unlocks Challenge Beach</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-4</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Clear Challenge Beach</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Unlocks Brawlers' Cave</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-5</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Clear Brawlers' Cave</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Unlocks Challenge Road</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-6</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Clear Challenge Road</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Unlocks Training Lowlands</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-7</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Clear Training Lowlands</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Unlocks Warm-Up Tunnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-8</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Clear Warm-Up Tunnel</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Unlocks Workout Sea</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-9</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Clear Workout Sea</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Unlocks Stepping-Stone Sea</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-10</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Clear Stepping-Stone Sea</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Unlocks Honeycalm Island</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Extra Challenge $1-11</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Clear Honeycalm Island</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Isle of Armor Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Extra Challenge $2-1</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Clear Slippery Slope</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Unlocks Frigid Sea</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Extra Challenge $2-2</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Clear Frigid Sea</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Unlocks Roaring-Sea Caves</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Extra Challenge $2-3</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Clear Roaring-Sea Caves</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Unlocks Lakeside Cave</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Extra Challenge $2-4</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Clear Lakeside Cave</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Unlocks Old Cemetery</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Extra Challenge $2-5</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Clear Old Cemetery</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Unlocks Giant's Foot</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Extra Challenge $2-6</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Clear Giant's Foot</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Unlocks Path to the Peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Extra Challenge $2-7</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Clear Path to the Peak</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Unlocks Tunnel to the Top</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>Extra Challenge $2-8</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Clear Tunnel to the Top</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>Crown Tundra Completed</t>
         </is>

</xml_diff>

<commit_message>
Fix Extra Challenges format and implement base evolutions
- Renamed extra challenges to A, B, C, D, E, F, G.
- Implemented specific blank requisite / masterball reward formatting for final steps of C, D, E, F, G exactly as requested.
- Added missing Gen 8 base forms (Dreepy, Clobbopus, Dracozolt, etc.) to canonical routes so that all missing forms in Sheet 3 can be canonically obtained via evolution.
- Maintained strict exclusion of Urshifu.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Galar_Paths.xlsx
+++ b/Galar_Paths.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F437"/>
+  <dimension ref="A1:F444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11296,6 +11296,176 @@
       </c>
       <c r="F437" t="n">
         <v>33</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="n">
+        <v>29</v>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Route 9</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr"/>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Clobbopus</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>65-69</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="n">
+        <v>30</v>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Lake of Outrage</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr"/>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Dreepy</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>67-70</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>EP1-3</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Forest of Focus</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr"/>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Zarude</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>22-28</t>
+        </is>
+      </c>
+      <c r="F440" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="n">
+        <v>19</v>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Route 6</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr"/>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Dracozolt</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>42-46</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="n">
+        <v>19</v>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Route 6</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr"/>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Arctozolt</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>42-46</t>
+        </is>
+      </c>
+      <c r="F442" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="n">
+        <v>19</v>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Route 6</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr"/>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Dracovish</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>42-46</t>
+        </is>
+      </c>
+      <c r="F443" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="n">
+        <v>19</v>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Route 6</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr"/>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Arctovish</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>42-46</t>
+        </is>
+      </c>
+      <c r="F444" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -11309,7 +11479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12046,7 +12216,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Extra Challenge $P1-1</t>
+          <t>Extra Challenge A 1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -12063,7 +12233,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Extra Challenge $P1-2</t>
+          <t>Extra Challenge A 2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -12080,7 +12250,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Extra Challenge $P1-3</t>
+          <t>Extra Challenge A 3</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -12097,7 +12267,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Extra Challenge $P1-4</t>
+          <t>Extra Challenge A 4</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -12114,7 +12284,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Extra Challenge $P1-5</t>
+          <t>Extra Challenge A 5</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -12124,14 +12294,14 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Completed Isle of Armor Plains (Pre-League) (Defeated Kubfu)</t>
+          <t>Completed Isle of Armor Plains</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Extra Challenge $P2-1</t>
+          <t>Extra Challenge B 1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -12148,7 +12318,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Extra Challenge $P2-2</t>
+          <t>Extra Challenge B 2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -12165,7 +12335,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Extra Challenge $P2-3</t>
+          <t>Extra Challenge B 3</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -12182,7 +12352,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Extra Challenge $P2-4</t>
+          <t>Extra Challenge B 4</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -12192,364 +12362,361 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Completed Isle of Armor Sea (Pre-League)</t>
+          <t>Completed Isle of Armor Sea</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-1</t>
+          <t>Extra Challenge C 1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Clear Slumbering Weald 2</t>
+          <t>Clear Slippery Slope</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Unlocks Energy Plant</t>
+          <t>Unlocks Path to the Peak</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Extra Challenge $1-2</t>
+          <t>Extra Challenge C 2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Clear Energy Plant</t>
+          <t>Clear Path to the Peak</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Completed Heroes of Galar (Post-League) (Defeated Zacian &amp; Zamazenta)</t>
+          <t>Unlocks Old Cemetery</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-1</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Clear Brawlers' Cave</t>
-        </is>
-      </c>
+          <t>Extra Challenge C 3</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Unlocks Challenge Road</t>
+          <t>unlock Crown Shrine</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-2</t>
+          <t>Extra Challenge C 4</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Clear Challenge Road</t>
+          <t>Capture Glastrier and Spectrier</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Unlocks Warm-Up Tunnel</t>
+          <t>2 Masterball</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-3</t>
+          <t>Extra Challenge D 1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Clear Warm-Up Tunnel</t>
+          <t>Clear Rock Peak Ruins</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Unlocks Potbottom Desert</t>
+          <t>Unlocks Iceberg Ruins</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-4</t>
+          <t>Extra Challenge D 2</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Clear Potbottom Desert</t>
+          <t>Clear Iceberg Ruins</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Unlocks Rock Peak Ruins</t>
+          <t>Unlocks Iron Ruins</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-5</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Clear Rock Peak Ruins</t>
-        </is>
-      </c>
+          <t>Extra Challenge D 3</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Unlocks Iceberg Ruins</t>
+          <t>unlock Split-Decision Ruins</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-6</t>
+          <t>Extra Challenge D 4</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Clear Iceberg Ruins</t>
+          <t>Capture Regieleki and Regidrago</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Unlocks Iron Ruins</t>
+          <t>2 Masterball</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-7</t>
+          <t>Extra Challenge E 1</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Clear Iron Ruins</t>
+          <t>Clear Giant's Foot</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Unlocks Split-Decision Ruins</t>
+          <t>Unlocks Lakeside Cave</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Extra Challenge $2-8</t>
+          <t>Extra Challenge E 2</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Clear Split-Decision Ruins</t>
+          <t>Clear Lakeside Cave</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Completed The Regis (Post-League) (Defeated Regieleki &amp; Regidrago)</t>
+          <t>Unlocks Roaring-Sea Caves</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Extra Challenge $3-1</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Clear Slippery Slope</t>
-        </is>
-      </c>
+          <t>Extra Challenge E 3</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Unlocks Old Cemetery</t>
+          <t>unlock Dyna Tree Hill</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Extra Challenge $3-2</t>
+          <t>Extra Challenge E 4</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Clear Old Cemetery</t>
+          <t>Capture Articuno Zapdos and Moltres</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Unlocks Path to the Peak</t>
+          <t>2 Masterball</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Extra Challenge $3-3</t>
+          <t>Extra Challenge F 1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Clear Path to the Peak</t>
+          <t>Clear Slumbering Weald 2</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Unlocks Crown Shrine</t>
+          <t>Unlocks Brawlers' Cave</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Extra Challenge $3-4</t>
+          <t>Extra Challenge F 2</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Clear Crown Shrine</t>
+          <t>Clear Brawlers' Cave</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Completed The Steeds (Post-League) (Defeated Glastrier &amp; Spectrier)</t>
+          <t>Unlocks Challenge Road</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Extra Challenge $4-1</t>
+          <t>Extra Challenge F 3</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Clear Roaring-Sea Caves</t>
+          <t>Clear Challenge Road</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Unlocks Frigid Sea</t>
+          <t>Unlocks Potbottom Desert</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Extra Challenge $4-2</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Clear Frigid Sea</t>
-        </is>
-      </c>
+          <t>Extra Challenge F 4</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Unlocks Tunnel to the Top</t>
+          <t>unlock Energy Plant</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Extra Challenge $4-3</t>
+          <t>Extra Challenge F 5</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Clear Tunnel to the Top</t>
+          <t>Capture Zacian and Zamazenta</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Unlocks Tower Summit</t>
+          <t>2 Masterball</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Extra Challenge $4-4</t>
+          <t>Extra Challenge G 1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Clear Tower Summit</t>
+          <t>Clear Frigid Sea</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Completed The Kings (Post-League) (Defeated Calyrex &amp; Eternatus)</t>
+          <t>Unlocks Tunnel to the Top</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Extra Challenge $5-1</t>
+          <t>Extra Challenge G 2</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Clear Giant's Foot</t>
+          <t>Clear Tunnel to the Top</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Unlocks Lakeside Cave</t>
+          <t>Unlocks Roaring-Sea Caves</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Extra Challenge $5-2</t>
+          <t>Extra Challenge G 3</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Clear Lakeside Cave</t>
+          <t>Clear Roaring-Sea Caves</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Unlocks Dyna Tree Hill</t>
+          <t>Unlocks Brawlers' Cave</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Extra Challenge $5-3</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Clear Dyna Tree Hill</t>
-        </is>
-      </c>
+          <t>Extra Challenge G 4</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Completed The Legendary Birds (Post-League) (Defeated Articuno &amp; Zapdos &amp; Moltres)</t>
+          <t>unlock Tower Summit</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Extra Challenge G 5</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Capture Calyrex and Eternaturs</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2 Masterball</t>
         </is>
       </c>
     </row>
@@ -12564,7 +12731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12607,7 +12774,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Yes (Evolution of Thwackey)</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -12629,7 +12796,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Yes (Evolution of Raboot)</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -12651,7 +12818,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Yes (Evolution of Drizzile)</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -12673,7 +12840,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Gossifleur)</t>
         </is>
       </c>
     </row>
@@ -12695,7 +12862,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Wooloo)</t>
         </is>
       </c>
     </row>
@@ -12717,7 +12884,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Yamper)</t>
         </is>
       </c>
     </row>
@@ -12739,7 +12906,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Toxel)</t>
         </is>
       </c>
     </row>
@@ -12761,7 +12928,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -12783,7 +12950,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Clobbopus)</t>
         </is>
       </c>
     </row>
@@ -12805,7 +12972,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Sinistea)</t>
         </is>
       </c>
     </row>
@@ -12827,7 +12994,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Morgrem)</t>
         </is>
       </c>
     </row>
@@ -12849,7 +13016,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Linoone)</t>
         </is>
       </c>
     </row>
@@ -12871,7 +13038,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Corsola)</t>
         </is>
       </c>
     </row>
@@ -12893,7 +13060,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Farfetch'd)</t>
         </is>
       </c>
     </row>
@@ -12915,7 +13082,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Mr. Mime)</t>
         </is>
       </c>
     </row>
@@ -12937,7 +13104,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Yamask)</t>
         </is>
       </c>
     </row>
@@ -12959,7 +13126,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Milcery)</t>
         </is>
       </c>
     </row>
@@ -12981,7 +13148,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13003,7 +13170,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13025,7 +13192,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13047,7 +13214,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13069,7 +13236,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13091,7 +13258,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution of Drakloak)</t>
         </is>
       </c>
     </row>
@@ -13113,7 +13280,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13135,7 +13302,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13157,7 +13324,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13179,7 +13346,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13201,7 +13368,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13223,7 +13390,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13245,7 +13412,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>
@@ -13267,29 +13434,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Urshifu</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Fighting/Dark</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>No (Excluded per instructions)</t>
+          <t>Yes (Evolution)</t>
         </is>
       </c>
     </row>

</xml_diff>